<commit_message>
Gel 2 egalites : complément de Léo (ecart_emploi_fh hors socle), 9 décisions ; D48 mis à jour
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015bc6mL53Gt9fSuWNDrxWfS
</commit_message>
<xml_diff>
--- a/docs/validation/classeurs/retours/validation_egalites_2026-10-17.xlsx
+++ b/docs/validation/classeurs/retours/validation_egalites_2026-10-17.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LMalherbe\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/769b183d86f89f3a/Recherche/Projets/Observatoire de la prospérité/Prosperity x Claude/30_dimensions_indicateurs/validation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F89E8AC0-CF13-4FCF-90A7-3AA7E1BBA778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{F89E8AC0-CF13-4FCF-90A7-3AA7E1BBA778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60FEB555-A46B-4946-8CAF-4DBED083568E}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1034" uniqueCount="482">
   <si>
     <t>Gel 2 — validation des indicateurs de la dimension « Égalités »</t>
   </si>
@@ -2865,7 +2865,9 @@
       <c r="Q15" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="R15" s="7"/>
+      <c r="R15" s="7" t="s">
+        <v>50</v>
+      </c>
       <c r="S15" s="7"/>
     </row>
     <row r="16" spans="1:19" ht="60" customHeight="1" x14ac:dyDescent="0.35">
@@ -5396,7 +5398,7 @@
       </c>
       <c r="B16" s="9">
         <f>COUNTA(Validation!$R$2:$R$58)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -5414,7 +5416,7 @@
       </c>
       <c r="B18" s="9">
         <f>COUNTIF(Validation!$R$2:$R$58,"retenu")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>